<commit_message>
Atualiza bases: filtro de canais, cruzamento NFD x Intelipost corrigido, cache de cotacao
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -396,10 +396,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2">
-        <v>733884</v>
+        <v>683650</v>
       </c>
       <c r="B2">
-        <v>506836155.5899999</v>
+        <v>159669864.86</v>
       </c>
       <c r="C2">
         <v>0</v>

</xml_diff>

<commit_message>
Atualizacao Regras PRW + Impacto Financeiro
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>TotalPedidos</t>
   </si>
@@ -23,6 +23,15 @@
   </si>
   <si>
     <t>PedidosSemValorNota</t>
+  </si>
+  <si>
+    <t>TotalVendasBruto</t>
+  </si>
+  <si>
+    <t>TotalNFDBruto</t>
+  </si>
+  <si>
+    <t>NFDSemTransportadora</t>
   </si>
 </sst>
 </file>
@@ -380,10 +389,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -393,8 +402,17 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>683650</v>
       </c>
@@ -403,6 +421,15 @@
       </c>
       <c r="C2">
         <v>0</v>
+      </c>
+      <c r="D2">
+        <v>175928860.3900001</v>
+      </c>
+      <c r="E2">
+        <v>11800460.23</v>
+      </c>
+      <c r="F2">
+        <v>52388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ETL atualizado: TspMasNaoTsp e CruzouIntelipost propagados para base do site
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -414,22 +414,22 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2">
-        <v>683650</v>
+        <v>862530</v>
       </c>
       <c r="B2">
-        <v>159669864.86</v>
+        <v>197488916.1900001</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>175928860.3900001</v>
+        <v>204513156.83</v>
       </c>
       <c r="E2">
-        <v>11800460.23</v>
+        <v>12736795.36</v>
       </c>
       <c r="F2">
-        <v>21883</v>
+        <v>27460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ETL: NFD sem transportadora corrigido para 14693 com fallback PRW
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>TotalPedidos</t>
   </si>
@@ -32,6 +32,12 @@
   </si>
   <si>
     <t>NFDSemTransportadora</t>
+  </si>
+  <si>
+    <t>NFDTranspIntelipost</t>
+  </si>
+  <si>
+    <t>NFDTranspPRWFallback</t>
   </si>
 </sst>
 </file>
@@ -389,10 +395,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -411,8 +417,14 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>862530</v>
       </c>
@@ -429,7 +441,13 @@
         <v>12736795.36</v>
       </c>
       <c r="F2">
-        <v>27460</v>
+        <v>14693</v>
+      </c>
+      <c r="G2">
+        <v>33175</v>
+      </c>
+      <c r="H2">
+        <v>12767</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ETL+App: NFD sem transportadora TSP corrigido para 602
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>TotalPedidos</t>
   </si>
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>NFDSemTransportadora</t>
+  </si>
+  <si>
+    <t>NFDSemTransportadoraTSP</t>
   </si>
   <si>
     <t>NFDTranspIntelipost</t>
@@ -395,10 +398,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -423,8 +426,11 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2">
         <v>862530</v>
       </c>
@@ -444,9 +450,12 @@
         <v>14693</v>
       </c>
       <c r="G2">
+        <v>602</v>
+      </c>
+      <c r="H2">
         <v>33175</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>12767</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ETL: corrige cache Rentabilidade (duplicacao), formula ganho liquido, NFD sem transportadora
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>TotalPedidos</t>
   </si>
@@ -32,9 +32,6 @@
   </si>
   <si>
     <t>NFDSemTransportadora</t>
-  </si>
-  <si>
-    <t>NFDSemTransportadoraTSP</t>
   </si>
   <si>
     <t>NFDTranspIntelipost</t>
@@ -398,10 +395,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -426,11 +423,8 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>862530</v>
       </c>
@@ -441,22 +435,19 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>204513156.83</v>
+        <v>240176319.35</v>
       </c>
       <c r="E2">
-        <v>12736795.36</v>
+        <v>13043610.06</v>
       </c>
       <c r="F2">
-        <v>14693</v>
+        <v>15138</v>
       </c>
       <c r="G2">
-        <v>602</v>
+        <v>33636</v>
       </c>
       <c r="H2">
-        <v>33175</v>
-      </c>
-      <c r="I2">
-        <v>12767</v>
+        <v>12847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ETL: corrige cache Rentabilidade, formula ganho liquido, NFD sem transportadora
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -435,19 +435,19 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>240176319.35</v>
+        <v>282414297.3600001</v>
       </c>
       <c r="E2">
-        <v>13043610.06</v>
+        <v>13387004.75</v>
       </c>
       <c r="F2">
-        <v>15138</v>
+        <v>15262</v>
       </c>
       <c r="G2">
-        <v>33636</v>
+        <v>34550</v>
       </c>
       <c r="H2">
-        <v>12847</v>
+        <v>13524</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao Monitor (upload web)
</commit_message>
<xml_diff>
--- a/data/Base_Intelipost_Resumo.xlsx
+++ b/data/Base_Intelipost_Resumo.xlsx
@@ -432,10 +432,10 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2">
-        <v>1144654</v>
+        <v>1188159</v>
       </c>
       <c r="B2">
-        <v>254378835.0100001</v>
+        <v>263686820.63</v>
       </c>
       <c r="C2">
         <v>0</v>

</xml_diff>